<commit_message>
fix: ordenar lista da proxima fase
</commit_message>
<xml_diff>
--- a/templates/lista_15_selecionados_modelo.xlsx
+++ b/templates/lista_15_selecionados_modelo.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selecionados" sheetId="1" r:id="R61491446194243d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selecionados" sheetId="1" r:id="Rfa3c30f30f4e4af8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -245,12 +245,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -258,10 +258,10 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -270,10 +270,10 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -286,20 +286,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SelecionadosProximaFase" displayName="SelecionadosProximaFase" ref="A5:K20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K20"/>
-  <x:tableColumns count="11">
-    <x:tableColumn id="1" name="Posição"/>
-    <x:tableColumn id="2" name="ID"/>
-    <x:tableColumn id="3" name="Nome"/>
-    <x:tableColumn id="4" name="E-mail"/>
-    <x:tableColumn id="5" name="Idade"/>
-    <x:tableColumn id="6" name="Cidade"/>
-    <x:tableColumn id="7" name="Estado"/>
-    <x:tableColumn id="8" name="Região"/>
-    <x:tableColumn id="9" name="Gênero"/>
-    <x:tableColumn id="10" name="Raça"/>
-    <x:tableColumn id="11" name="Universidade"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SelecionadosProximaFase" displayName="SelecionadosProximaFase" ref="A5:J20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J20"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Nome"/>
+    <x:tableColumn id="3" name="E-mail"/>
+    <x:tableColumn id="4" name="Idade"/>
+    <x:tableColumn id="5" name="Cidade"/>
+    <x:tableColumn id="6" name="Estado"/>
+    <x:tableColumn id="7" name="Região"/>
+    <x:tableColumn id="8" name="Gênero"/>
+    <x:tableColumn id="9" name="Raça"/>
+    <x:tableColumn id="10" name="Universidade"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -503,17 +502,16 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="34" customHeight="1">
@@ -529,12 +527,9 @@
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4"/>
       <x:c r="J2" s="4"/>
-      <x:c r="K2" s="4"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="5" t="str">
-        <x:v>Lista das pessoas selecionadas, organizada no mesmo padrão da planilha de Marca Empregadora.</x:v>
-      </x:c>
+    </x:row>
+    <x:row r="3" ht="16" customHeight="1">
+      <x:c r="A3" s="5" t="str"/>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -544,7 +539,6 @@
       <x:c r="H3" s="1"/>
       <x:c r="I3" s="1"/>
       <x:c r="J3" s="1"/>
-      <x:c r="K3" s="1"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1"/>
@@ -557,246 +551,227 @@
       <x:c r="H4" s="1"/>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="1"/>
-      <x:c r="K4" s="1"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="16" t="str">
-        <x:v>Posição</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>ID</x:v>
+        <x:v>Nome</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>Nome</x:v>
+        <x:v>E-mail</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
-        <x:v>E-mail</x:v>
+        <x:v>Idade</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>Idade</x:v>
+        <x:v>Cidade</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>Cidade</x:v>
+        <x:v>Estado</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>Estado</x:v>
+        <x:v>Região</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>Região</x:v>
+        <x:v>Gênero</x:v>
       </x:c>
       <x:c r="I5" s="17" t="str">
-        <x:v>Gênero</x:v>
-      </x:c>
-      <x:c r="J5" s="17" t="str">
         <x:v>Raça</x:v>
       </x:c>
-      <x:c r="K5" s="18" t="str">
+      <x:c r="J5" s="18" t="str">
         <x:v>Universidade</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26" customHeight="1">
       <x:c r="A6" s="30" t="str"/>
       <x:c r="B6" s="31" t="str"/>
-      <x:c r="C6" s="32" t="str"/>
+      <x:c r="C6" s="31" t="str"/>
       <x:c r="D6" s="32" t="str"/>
-      <x:c r="E6" s="31" t="str"/>
-      <x:c r="F6" s="31" t="str"/>
-      <x:c r="G6" s="31" t="str"/>
-      <x:c r="H6" s="31" t="str"/>
-      <x:c r="I6" s="31" t="str"/>
-      <x:c r="J6" s="31" t="str"/>
-      <x:c r="K6" s="33" t="str"/>
+      <x:c r="E6" s="32" t="str"/>
+      <x:c r="F6" s="32" t="str"/>
+      <x:c r="G6" s="32" t="str"/>
+      <x:c r="H6" s="32" t="str"/>
+      <x:c r="I6" s="32" t="str"/>
+      <x:c r="J6" s="33" t="str"/>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="28" t="str"/>
-      <x:c r="B7" s="29" t="str"/>
+      <x:c r="A7" s="27" t="str"/>
+      <x:c r="B7" s="24" t="str"/>
       <x:c r="C7" s="24" t="str"/>
-      <x:c r="D7" s="24" t="str"/>
+      <x:c r="D7" s="29" t="str"/>
       <x:c r="E7" s="29" t="str"/>
       <x:c r="F7" s="29" t="str"/>
       <x:c r="G7" s="29" t="str"/>
       <x:c r="H7" s="29" t="str"/>
       <x:c r="I7" s="29" t="str"/>
-      <x:c r="J7" s="29" t="str"/>
-      <x:c r="K7" s="25" t="str"/>
+      <x:c r="J7" s="25" t="str"/>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
       <x:c r="A8" s="34" t="str"/>
       <x:c r="B8" s="35" t="str"/>
-      <x:c r="C8" s="36" t="str"/>
+      <x:c r="C8" s="35" t="str"/>
       <x:c r="D8" s="36" t="str"/>
-      <x:c r="E8" s="35" t="str"/>
-      <x:c r="F8" s="35" t="str"/>
-      <x:c r="G8" s="35" t="str"/>
-      <x:c r="H8" s="35" t="str"/>
-      <x:c r="I8" s="35" t="str"/>
-      <x:c r="J8" s="35" t="str"/>
-      <x:c r="K8" s="37" t="str"/>
+      <x:c r="E8" s="36" t="str"/>
+      <x:c r="F8" s="36" t="str"/>
+      <x:c r="G8" s="36" t="str"/>
+      <x:c r="H8" s="36" t="str"/>
+      <x:c r="I8" s="36" t="str"/>
+      <x:c r="J8" s="37" t="str"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="28" t="str"/>
-      <x:c r="B9" s="29" t="str"/>
+      <x:c r="A9" s="27" t="str"/>
+      <x:c r="B9" s="24" t="str"/>
       <x:c r="C9" s="24" t="str"/>
-      <x:c r="D9" s="24" t="str"/>
+      <x:c r="D9" s="29" t="str"/>
       <x:c r="E9" s="29" t="str"/>
       <x:c r="F9" s="29" t="str"/>
       <x:c r="G9" s="29" t="str"/>
       <x:c r="H9" s="29" t="str"/>
       <x:c r="I9" s="29" t="str"/>
-      <x:c r="J9" s="29" t="str"/>
-      <x:c r="K9" s="25" t="str"/>
+      <x:c r="J9" s="25" t="str"/>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
       <x:c r="A10" s="34" t="str"/>
       <x:c r="B10" s="35" t="str"/>
-      <x:c r="C10" s="36" t="str"/>
+      <x:c r="C10" s="35" t="str"/>
       <x:c r="D10" s="36" t="str"/>
-      <x:c r="E10" s="35" t="str"/>
-      <x:c r="F10" s="35" t="str"/>
-      <x:c r="G10" s="35" t="str"/>
-      <x:c r="H10" s="35" t="str"/>
-      <x:c r="I10" s="35" t="str"/>
-      <x:c r="J10" s="35" t="str"/>
-      <x:c r="K10" s="37" t="str"/>
+      <x:c r="E10" s="36" t="str"/>
+      <x:c r="F10" s="36" t="str"/>
+      <x:c r="G10" s="36" t="str"/>
+      <x:c r="H10" s="36" t="str"/>
+      <x:c r="I10" s="36" t="str"/>
+      <x:c r="J10" s="37" t="str"/>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
-      <x:c r="A11" s="28" t="str"/>
-      <x:c r="B11" s="29" t="str"/>
+      <x:c r="A11" s="27" t="str"/>
+      <x:c r="B11" s="24" t="str"/>
       <x:c r="C11" s="24" t="str"/>
-      <x:c r="D11" s="24" t="str"/>
+      <x:c r="D11" s="29" t="str"/>
       <x:c r="E11" s="29" t="str"/>
       <x:c r="F11" s="29" t="str"/>
       <x:c r="G11" s="29" t="str"/>
       <x:c r="H11" s="29" t="str"/>
       <x:c r="I11" s="29" t="str"/>
-      <x:c r="J11" s="29" t="str"/>
-      <x:c r="K11" s="25" t="str"/>
+      <x:c r="J11" s="25" t="str"/>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">
       <x:c r="A12" s="34" t="str"/>
       <x:c r="B12" s="35" t="str"/>
-      <x:c r="C12" s="36" t="str"/>
+      <x:c r="C12" s="35" t="str"/>
       <x:c r="D12" s="36" t="str"/>
-      <x:c r="E12" s="35" t="str"/>
-      <x:c r="F12" s="35" t="str"/>
-      <x:c r="G12" s="35" t="str"/>
-      <x:c r="H12" s="35" t="str"/>
-      <x:c r="I12" s="35" t="str"/>
-      <x:c r="J12" s="35" t="str"/>
-      <x:c r="K12" s="37" t="str"/>
+      <x:c r="E12" s="36" t="str"/>
+      <x:c r="F12" s="36" t="str"/>
+      <x:c r="G12" s="36" t="str"/>
+      <x:c r="H12" s="36" t="str"/>
+      <x:c r="I12" s="36" t="str"/>
+      <x:c r="J12" s="37" t="str"/>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
-      <x:c r="A13" s="28" t="str"/>
-      <x:c r="B13" s="29" t="str"/>
+      <x:c r="A13" s="27" t="str"/>
+      <x:c r="B13" s="24" t="str"/>
       <x:c r="C13" s="24" t="str"/>
-      <x:c r="D13" s="24" t="str"/>
+      <x:c r="D13" s="29" t="str"/>
       <x:c r="E13" s="29" t="str"/>
       <x:c r="F13" s="29" t="str"/>
       <x:c r="G13" s="29" t="str"/>
       <x:c r="H13" s="29" t="str"/>
       <x:c r="I13" s="29" t="str"/>
-      <x:c r="J13" s="29" t="str"/>
-      <x:c r="K13" s="25" t="str"/>
+      <x:c r="J13" s="25" t="str"/>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
       <x:c r="A14" s="34" t="str"/>
       <x:c r="B14" s="35" t="str"/>
-      <x:c r="C14" s="36" t="str"/>
+      <x:c r="C14" s="35" t="str"/>
       <x:c r="D14" s="36" t="str"/>
-      <x:c r="E14" s="35" t="str"/>
-      <x:c r="F14" s="35" t="str"/>
-      <x:c r="G14" s="35" t="str"/>
-      <x:c r="H14" s="35" t="str"/>
-      <x:c r="I14" s="35" t="str"/>
-      <x:c r="J14" s="35" t="str"/>
-      <x:c r="K14" s="37" t="str"/>
+      <x:c r="E14" s="36" t="str"/>
+      <x:c r="F14" s="36" t="str"/>
+      <x:c r="G14" s="36" t="str"/>
+      <x:c r="H14" s="36" t="str"/>
+      <x:c r="I14" s="36" t="str"/>
+      <x:c r="J14" s="37" t="str"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="28" t="str"/>
-      <x:c r="B15" s="29" t="str"/>
+      <x:c r="A15" s="27" t="str"/>
+      <x:c r="B15" s="24" t="str"/>
       <x:c r="C15" s="24" t="str"/>
-      <x:c r="D15" s="24" t="str"/>
+      <x:c r="D15" s="29" t="str"/>
       <x:c r="E15" s="29" t="str"/>
       <x:c r="F15" s="29" t="str"/>
       <x:c r="G15" s="29" t="str"/>
       <x:c r="H15" s="29" t="str"/>
       <x:c r="I15" s="29" t="str"/>
-      <x:c r="J15" s="29" t="str"/>
-      <x:c r="K15" s="25" t="str"/>
+      <x:c r="J15" s="25" t="str"/>
     </x:row>
     <x:row r="16" ht="26" customHeight="1">
       <x:c r="A16" s="34" t="str"/>
       <x:c r="B16" s="35" t="str"/>
-      <x:c r="C16" s="36" t="str"/>
+      <x:c r="C16" s="35" t="str"/>
       <x:c r="D16" s="36" t="str"/>
-      <x:c r="E16" s="35" t="str"/>
-      <x:c r="F16" s="35" t="str"/>
-      <x:c r="G16" s="35" t="str"/>
-      <x:c r="H16" s="35" t="str"/>
-      <x:c r="I16" s="35" t="str"/>
-      <x:c r="J16" s="35" t="str"/>
-      <x:c r="K16" s="37" t="str"/>
+      <x:c r="E16" s="36" t="str"/>
+      <x:c r="F16" s="36" t="str"/>
+      <x:c r="G16" s="36" t="str"/>
+      <x:c r="H16" s="36" t="str"/>
+      <x:c r="I16" s="36" t="str"/>
+      <x:c r="J16" s="37" t="str"/>
     </x:row>
     <x:row r="17" ht="26" customHeight="1">
-      <x:c r="A17" s="28" t="str"/>
-      <x:c r="B17" s="29" t="str"/>
+      <x:c r="A17" s="27" t="str"/>
+      <x:c r="B17" s="24" t="str"/>
       <x:c r="C17" s="24" t="str"/>
-      <x:c r="D17" s="24" t="str"/>
+      <x:c r="D17" s="29" t="str"/>
       <x:c r="E17" s="29" t="str"/>
       <x:c r="F17" s="29" t="str"/>
       <x:c r="G17" s="29" t="str"/>
       <x:c r="H17" s="29" t="str"/>
       <x:c r="I17" s="29" t="str"/>
-      <x:c r="J17" s="29" t="str"/>
-      <x:c r="K17" s="25" t="str"/>
+      <x:c r="J17" s="25" t="str"/>
     </x:row>
     <x:row r="18" ht="26" customHeight="1">
       <x:c r="A18" s="34" t="str"/>
       <x:c r="B18" s="35" t="str"/>
-      <x:c r="C18" s="36" t="str"/>
+      <x:c r="C18" s="35" t="str"/>
       <x:c r="D18" s="36" t="str"/>
-      <x:c r="E18" s="35" t="str"/>
-      <x:c r="F18" s="35" t="str"/>
-      <x:c r="G18" s="35" t="str"/>
-      <x:c r="H18" s="35" t="str"/>
-      <x:c r="I18" s="35" t="str"/>
-      <x:c r="J18" s="35" t="str"/>
-      <x:c r="K18" s="37" t="str"/>
+      <x:c r="E18" s="36" t="str"/>
+      <x:c r="F18" s="36" t="str"/>
+      <x:c r="G18" s="36" t="str"/>
+      <x:c r="H18" s="36" t="str"/>
+      <x:c r="I18" s="36" t="str"/>
+      <x:c r="J18" s="37" t="str"/>
     </x:row>
     <x:row r="19" ht="26" customHeight="1">
-      <x:c r="A19" s="28" t="str"/>
-      <x:c r="B19" s="29" t="str"/>
+      <x:c r="A19" s="27" t="str"/>
+      <x:c r="B19" s="24" t="str"/>
       <x:c r="C19" s="24" t="str"/>
-      <x:c r="D19" s="24" t="str"/>
+      <x:c r="D19" s="29" t="str"/>
       <x:c r="E19" s="29" t="str"/>
       <x:c r="F19" s="29" t="str"/>
       <x:c r="G19" s="29" t="str"/>
       <x:c r="H19" s="29" t="str"/>
       <x:c r="I19" s="29" t="str"/>
-      <x:c r="J19" s="29" t="str"/>
-      <x:c r="K19" s="25" t="str"/>
+      <x:c r="J19" s="25" t="str"/>
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
       <x:c r="A20" s="34" t="str"/>
       <x:c r="B20" s="35" t="str"/>
-      <x:c r="C20" s="36" t="str"/>
+      <x:c r="C20" s="35" t="str"/>
       <x:c r="D20" s="36" t="str"/>
-      <x:c r="E20" s="35" t="str"/>
-      <x:c r="F20" s="35" t="str"/>
-      <x:c r="G20" s="35" t="str"/>
-      <x:c r="H20" s="35" t="str"/>
-      <x:c r="I20" s="35" t="str"/>
-      <x:c r="J20" s="35" t="str"/>
-      <x:c r="K20" s="37" t="str"/>
+      <x:c r="E20" s="36" t="str"/>
+      <x:c r="F20" s="36" t="str"/>
+      <x:c r="G20" s="36" t="str"/>
+      <x:c r="H20" s="36" t="str"/>
+      <x:c r="I20" s="36" t="str"/>
+      <x:c r="J20" s="37" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:K2"/>
-    <x:mergeCell ref="A3:K3"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A3:J3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R007b1a0df35a4f25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08b1b616809c4990"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>